<commit_message>
Update README with benchmarking results and features
</commit_message>
<xml_diff>
--- a/results/hyperparameter_results.xlsx
+++ b/results/hyperparameter_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,7 +434,92 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Hidden</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Dropout</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Weight_Decay</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Epochs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Macro_F1</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Weighted_F1</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Training_Time</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Parameters</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Memory_MB</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>AUC</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Average_Precision</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Hits@K</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Common_Neighbors</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Adamic_Adar</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Preferential_Attachment</t>
         </is>
       </c>
     </row>
@@ -455,8 +540,45 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.8110000000000001</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H2" t="n">
+        <v>200</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.749</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.7472</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.7484</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="M2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="N2" t="n">
+        <v>373.26</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -475,8 +597,45 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8090000000000001</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H3" t="n">
+        <v>200</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.7624</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.7727000000000001</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="M3" t="n">
+        <v>92359</v>
+      </c>
+      <c r="N3" t="n">
+        <v>380.09</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -495,8 +654,45 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8080000000000001</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H4" t="n">
+        <v>200</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.723</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.7238</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.7217</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="M4" t="n">
+        <v>46183</v>
+      </c>
+      <c r="N4" t="n">
+        <v>374.39</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -515,13 +711,50 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.794</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H5" t="n">
+        <v>200</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.752</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.7546</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.7502</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="M5" t="n">
+        <v>46183</v>
+      </c>
+      <c r="N5" t="n">
+        <v>374.57</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>link</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -535,13 +768,58 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.803</v>
+        <v>32</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H6" t="n">
+        <v>200</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="M6" t="n">
+        <v>47008</v>
+      </c>
+      <c r="N6" t="n">
+        <v>383.25</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.7786</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.7926</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.7271</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.6445</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>link</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -555,13 +833,58 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.8110000000000001</v>
+        <v>64</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H7" t="n">
+        <v>200</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="M7" t="n">
+        <v>96064</v>
+      </c>
+      <c r="N7" t="n">
+        <v>389.09</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.7901</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.8053</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.7196</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.6526</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>link</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -575,13 +898,58 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.8110000000000001</v>
+        <v>32</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H8" t="n">
+        <v>200</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="M8" t="n">
+        <v>47008</v>
+      </c>
+      <c r="N8" t="n">
+        <v>383.34</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.7685999999999999</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.7763</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.7181</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.6431</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>link</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -595,13 +963,58 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.8110000000000001</v>
+        <v>32</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H9" t="n">
+        <v>200</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="M9" t="n">
+        <v>47008</v>
+      </c>
+      <c r="N9" t="n">
+        <v>382.21</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.7473</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.7478</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.7036</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.6384</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>graph</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -611,17 +1024,52 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>cora</t>
+          <t>mutag</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.8</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H10" t="n">
+        <v>200</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.7389 ± 0.0975</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>40.36</v>
+      </c>
+      <c r="M10" t="n">
+        <v>386</v>
+      </c>
+      <c r="N10" t="n">
+        <v>362.55</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>graph</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -631,17 +1079,52 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>cora</t>
+          <t>mutag</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.8110000000000001</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H11" t="n">
+        <v>200</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.7228 ± 0.0995</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>43.63</v>
+      </c>
+      <c r="M11" t="n">
+        <v>770</v>
+      </c>
+      <c r="N11" t="n">
+        <v>365.25</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>graph</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -651,17 +1134,52 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>cora</t>
+          <t>mutag</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.8070000000000001</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H12" t="n">
+        <v>200</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.7336 ± 0.1043</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>40.26</v>
+      </c>
+      <c r="M12" t="n">
+        <v>386</v>
+      </c>
+      <c r="N12" t="n">
+        <v>361.62</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>graph</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -671,12 +1189,47 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>cora</t>
+          <t>mutag</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.8110000000000001</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H13" t="n">
+        <v>200</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.7284 ± 0.085</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>386</v>
+      </c>
+      <c r="N13" t="n">
+        <v>363.03</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -695,8 +1248,450 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.8070000000000001</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H14" t="n">
+        <v>200</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.7403999999999999</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.7425</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="M14" t="n">
+        <v>46183</v>
+      </c>
+      <c r="N14" t="n">
+        <v>373.91</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>gcn</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>cora</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>32</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H15" t="n">
+        <v>200</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="M15" t="n">
+        <v>47008</v>
+      </c>
+      <c r="N15" t="n">
+        <v>382.77</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.7755</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.7868000000000001</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.7252</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>graph</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gcn</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>mutag</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>32</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H16" t="n">
+        <v>200</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.7178 ± 0.0897</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>40.24</v>
+      </c>
+      <c r="M16" t="n">
+        <v>386</v>
+      </c>
+      <c r="N16" t="n">
+        <v>361.89</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>gcn</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>cora</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>32</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H17" t="n">
+        <v>200</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.749</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.7472</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.7484</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="M17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="N17" t="n">
+        <v>374.17</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>gat</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>cora</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>32</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H18" t="n">
+        <v>200</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.7711</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.7799</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>369941</v>
+      </c>
+      <c r="N18" t="n">
+        <v>473.73</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>graphsage</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>cora</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>32</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H19" t="n">
+        <v>200</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.7647</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.7742</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M19" t="n">
+        <v>92263</v>
+      </c>
+      <c r="N19" t="n">
+        <v>470.38</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>gin</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>cora</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>32</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H20" t="n">
+        <v>200</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.7496</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.7556</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="M20" t="n">
+        <v>47239</v>
+      </c>
+      <c r="N20" t="n">
+        <v>453.52</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>gcn</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>citeseer</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H21" t="n">
+        <v>200</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.606</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.584</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.6177</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="M21" t="n">
+        <v>118790</v>
+      </c>
+      <c r="N21" t="n">
+        <v>406.91</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>